<commit_message>
Add support for macro-enabled documents (docm, pptm, xlsm) and update test files
</commit_message>
<xml_diff>
--- a/examples/output/phase3-interface-example.xlsx
+++ b/examples/output/phase3-interface-example.xlsx
@@ -2,6 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr date1904="false"/>
+  <bookViews>
+    <workbookView activeTab="0"/>
+  </bookViews>
   <sheets>
     <sheet name="Phase3" r:id="rId3" sheetId="1"/>
   </sheets>
@@ -97,13 +100,13 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s" s="1">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s" s="1">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s" s="1">
         <v>2</v>
       </c>
     </row>

</xml_diff>